<commit_message>
Switch commission model to 1% of booking/deal value
Replaces the flat placeholder EGP amounts with the confirmed 1%
commission rate, applied to both Sahel Reservation and Furnishing
Package tracks. Commission Due now computes as Booking/Deal Value x
rate instead of a fixed lookup.
</commit_message>
<xml_diff>
--- a/docs/nest-ambassadors/06-referral-tracking-sheet.xlsx
+++ b/docs/nest-ambassadors/06-referral-tracking-sheet.xlsx
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="153">
   <si>
     <t xml:space="preserve">Nest Ambassadors — Referral Tracking Workbook (V1)</t>
   </si>
@@ -112,7 +112,7 @@
     <t xml:space="preserve">•  Staff List — eligible Ambassadors, department, referral code. Feeds the Ambassador Name dropdown.</t>
   </si>
   <si>
-    <t xml:space="preserve">•  Commission Rules — flat EGP commission per product track. PLACEHOLDER VALUES — pending leadership sign-off per the Phase-0 decision (see 02-quick-win-action-plan.md).</t>
+    <t xml:space="preserve">•  Commission Rules — commission rate (1% of Booking/Deal Value) per product track, confirmed per the Phase-0 decision (see 02-quick-win-action-plan.md).</t>
   </si>
   <si>
     <t xml:space="preserve">•  Leaderboard — auto-computed per-Ambassador totals for the weekly WhatsApp broadcast.</t>
@@ -133,9 +133,6 @@
     <t xml:space="preserve">Placeholders to replace before launch</t>
   </si>
   <si>
-    <t xml:space="preserve">•  Commission amounts (Commission Rules tab) — pending the Phase-0 leadership decision.</t>
-  </si>
-  <si>
     <t xml:space="preserve">•  Staff List — replace the 10 sample employees with the real eligible-employee list from HR.</t>
   </si>
   <si>
@@ -475,16 +472,19 @@
     <t xml:space="preserve">Replace with the authoritative eligible-employee list from HR before launch.</t>
   </si>
   <si>
-    <t xml:space="preserve">Commission Amount (EGP)</t>
+    <t xml:space="preserve">Commission Rate (% of Booking/Deal Value)</t>
   </si>
   <si>
     <t xml:space="preserve">Status</t>
   </si>
   <si>
-    <t xml:space="preserve">PLACEHOLDER — pending Phase-0 leadership sign-off (L1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source: illustrative placeholder values for template purposes only. Real amounts must be sanity-checked against paid-media cost per booking and signed off by CCO/Commercial Director (see 02-quick-win-action-plan.md, decision L1).</t>
+    <t xml:space="preserve">Confirmed — 1% of booking value (L1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed — 1% of deal value (L1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: confirmed rate — 1% of Booking/Deal Value, both tracks. Commission Due in Referral Tracking = Booking/Deal Value x this rate. Edit the rate cells above if leadership revises it; Commission Due recalculates automatically.</t>
   </si>
   <si>
     <t xml:space="preserve">Referrals Submitted</t>
@@ -538,9 +538,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="#,##0&quot; EGP&quot;"/>
-    <numFmt numFmtId="166" formatCode="General"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0&quot; EGP&quot;"/>
+    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -736,10 +736,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -756,6 +752,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -768,15 +768,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1059,7 +1059,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
@@ -1173,11 +1173,6 @@
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1222,70 +1217,70 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="T1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="U1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="V1" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="V1" s="5" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1294,64 +1289,64 @@
         <v>REF-0001</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>47</v>
       </c>
       <c r="E2" s="6" t="str">
         <f aca="false">IFERROR(INDEX('Staff List'!$B$2:$B$11,MATCH(D2,'Staff List'!$A$2:$A$11,0)),"")</f>
         <v>Sales</v>
       </c>
       <c r="F2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="K2" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>53</v>
       </c>
       <c r="L2" s="6"/>
       <c r="M2" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="N2" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="O2" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="P2" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="Q2" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="Q2" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="R2" s="6" t="n">
         <v>185000</v>
       </c>
-      <c r="S2" s="7" t="n">
-        <f aca="false">IF(P2="Booked-Paid",IFERROR(INDEX('Commission Rules'!$B$2:$B$3,MATCH(J2,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
-        <v>1500</v>
+      <c r="S2" s="6" t="n">
+        <f aca="false">IF(P2="Booked-Paid",IFERROR(R2*INDEX('Commission Rules'!$B$2:$B$3,MATCH(J2,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
+        <v>1850</v>
       </c>
       <c r="T2" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="U2" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="U2" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="V2" s="6"/>
     </row>
@@ -1361,13 +1356,13 @@
         <v>REF-0002</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>63</v>
       </c>
       <c r="E3" s="6" t="str">
         <f aca="false">IFERROR(INDEX('Staff List'!$B$2:$B$11,MATCH(D3,'Staff List'!$A$2:$A$11,0)),"")</f>
@@ -1375,44 +1370,44 @@
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>65</v>
       </c>
       <c r="I3" s="6"/>
       <c r="J3" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="L3" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="M3" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="O3" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="M3" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="O3" s="6" t="s">
+      <c r="P3" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="Q3" s="6"/>
       <c r="R3" s="6"/>
       <c r="S3" s="6" t="str">
-        <f aca="false">IF(P3="Booked-Paid",IFERROR(INDEX('Commission Rules'!$B$2:$B$3,MATCH(J3,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
+        <f aca="false">IF(P3="Booked-Paid",IFERROR(R3*INDEX('Commission Rules'!$B$2:$B$3,MATCH(J3,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
         <v/>
       </c>
       <c r="T3" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="U3" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V3" s="6"/>
     </row>
@@ -1422,60 +1417,60 @@
         <v>REF-0003</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>72</v>
       </c>
       <c r="E4" s="6" t="str">
         <f aca="false">IFERROR(INDEX('Staff List'!$B$2:$B$11,MATCH(D4,'Staff List'!$A$2:$A$11,0)),"")</f>
         <v>Sales</v>
       </c>
       <c r="F4" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="L4" s="6"/>
       <c r="M4" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="N4" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="N4" s="6" t="s">
+      <c r="O4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="P4" s="6" t="s">
         <v>79</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="P4" s="6" t="s">
-        <v>80</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
       <c r="S4" s="6" t="str">
-        <f aca="false">IF(P4="Booked-Paid",IFERROR(INDEX('Commission Rules'!$B$2:$B$3,MATCH(J4,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
+        <f aca="false">IF(P4="Booked-Paid",IFERROR(R4*INDEX('Commission Rules'!$B$2:$B$3,MATCH(J4,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
         <v/>
       </c>
       <c r="T4" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="U4" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="V4" s="6"/>
     </row>
@@ -1485,13 +1480,13 @@
         <v>REF-0004</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E5" s="6" t="str">
         <f aca="false">IFERROR(INDEX('Staff List'!$B$2:$B$11,MATCH(D5,'Staff List'!$A$2:$A$11,0)),"")</f>
@@ -1499,50 +1494,50 @@
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="J5" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="J5" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="K5" s="6" t="s">
+      <c r="L5" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="L5" s="6" t="s">
+      <c r="M5" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q5" s="6" t="s">
         <v>86</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="O5" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="P5" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q5" s="6" t="s">
-        <v>87</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>210000</v>
       </c>
-      <c r="S5" s="7" t="n">
-        <f aca="false">IF(P5="Booked-Paid",IFERROR(INDEX('Commission Rules'!$B$2:$B$3,MATCH(J5,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
-        <v>1500</v>
+      <c r="S5" s="6" t="n">
+        <f aca="false">IF(P5="Booked-Paid",IFERROR(R5*INDEX('Commission Rules'!$B$2:$B$3,MATCH(J5,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
+        <v>2100</v>
       </c>
       <c r="T5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="U5" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="U5" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="V5" s="6"/>
     </row>
@@ -1552,54 +1547,54 @@
         <v>REF-0005</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="E6" s="6" t="str">
         <f aca="false">IFERROR(INDEX('Staff List'!$B$2:$B$11,MATCH(D6,'Staff List'!$A$2:$A$11,0)),"")</f>
         <v>Marketing</v>
       </c>
       <c r="F6" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>91</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>92</v>
       </c>
       <c r="I6" s="6"/>
       <c r="J6" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L6" s="6"/>
       <c r="M6" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N6" s="6"/>
       <c r="O6" s="6"/>
       <c r="P6" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
       <c r="S6" s="6" t="str">
-        <f aca="false">IF(P6="Booked-Paid",IFERROR(INDEX('Commission Rules'!$B$2:$B$3,MATCH(J6,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
+        <f aca="false">IF(P6="Booked-Paid",IFERROR(R6*INDEX('Commission Rules'!$B$2:$B$3,MATCH(J6,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
         <v/>
       </c>
       <c r="T6" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="U6" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V6" s="6"/>
     </row>
@@ -1609,13 +1604,13 @@
         <v>REF-0006</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="E7" s="6" t="str">
         <f aca="false">IFERROR(INDEX('Staff List'!$B$2:$B$11,MATCH(D7,'Staff List'!$A$2:$A$11,0)),"")</f>
@@ -1623,46 +1618,46 @@
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="I7" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="J7" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K7" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="J7" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="K7" s="6" t="s">
+      <c r="L7" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="L7" s="6" t="s">
+      <c r="M7" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="M7" s="6" t="s">
+      <c r="N7" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="N7" s="6" t="s">
-        <v>103</v>
-      </c>
       <c r="O7" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="Q7" s="6"/>
       <c r="R7" s="6"/>
       <c r="S7" s="6" t="str">
-        <f aca="false">IF(P7="Booked-Paid",IFERROR(INDEX('Commission Rules'!$B$2:$B$3,MATCH(J7,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
+        <f aca="false">IF(P7="Booked-Paid",IFERROR(R7*INDEX('Commission Rules'!$B$2:$B$3,MATCH(J7,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
         <v/>
       </c>
       <c r="T7" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="U7" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V7" s="6"/>
     </row>
@@ -1672,60 +1667,60 @@
         <v>REF-0007</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="E8" s="6" t="str">
         <f aca="false">IFERROR(INDEX('Staff List'!$B$2:$B$11,MATCH(D8,'Staff List'!$A$2:$A$11,0)),"")</f>
         <v>Marketing</v>
       </c>
       <c r="F8" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="G8" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="J8" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="K8" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="L8" s="6"/>
       <c r="M8" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Q8" s="6"/>
       <c r="R8" s="6"/>
       <c r="S8" s="6" t="str">
-        <f aca="false">IF(P8="Booked-Paid",IFERROR(INDEX('Commission Rules'!$B$2:$B$3,MATCH(J8,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
+        <f aca="false">IF(P8="Booked-Paid",IFERROR(R8*INDEX('Commission Rules'!$B$2:$B$3,MATCH(J8,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
         <v/>
       </c>
       <c r="T8" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="U8" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="V8" s="6"/>
     </row>
@@ -1735,13 +1730,13 @@
         <v>REF-0008</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E9" s="6" t="str">
         <f aca="false">IFERROR(INDEX('Staff List'!$B$2:$B$11,MATCH(D9,'Staff List'!$A$2:$A$11,0)),"")</f>
@@ -1749,48 +1744,48 @@
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>112</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>113</v>
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K9" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="L9" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="M9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="O9" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="P9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q9" s="6" t="s">
         <v>115</v>
-      </c>
-      <c r="M9" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="N9" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="O9" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="P9" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q9" s="6" t="s">
-        <v>116</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>195000</v>
       </c>
-      <c r="S9" s="7" t="n">
-        <f aca="false">IF(P9="Booked-Paid",IFERROR(INDEX('Commission Rules'!$B$2:$B$3,MATCH(J9,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
-        <v>1500</v>
+      <c r="S9" s="6" t="n">
+        <f aca="false">IF(P9="Booked-Paid",IFERROR(R9*INDEX('Commission Rules'!$B$2:$B$3,MATCH(J9,'Commission Rules'!$A$2:$A$3,0)),""),"")</f>
+        <v>1950</v>
       </c>
       <c r="T9" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="U9" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="U9" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="V9" s="6"/>
     </row>
@@ -1880,161 +1875,161 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>27</v>
-      </c>
       <c r="C1" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>48</v>
-      </c>
       <c r="D2" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>73</v>
-      </c>
       <c r="D3" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>90</v>
-      </c>
       <c r="D6" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>106</v>
-      </c>
       <c r="D7" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>124</v>
-      </c>
       <c r="D8" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>126</v>
-      </c>
       <c r="D9" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="C10" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>129</v>
-      </c>
       <c r="D10" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="D11" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>132</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2057,49 +2052,49 @@
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2" s="9" t="n">
-        <v>1500</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>136</v>
+        <v>51</v>
+      </c>
+      <c r="B2" s="8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="9" t="n">
-        <v>800</v>
-      </c>
-      <c r="C3" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2131,10 +2126,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>27</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>138</v>
@@ -2170,9 +2165,9 @@
         <f aca="false">COUNTIFS('Referral Tracking'!$D$2:$D$500,A2,'Referral Tracking'!$P$2:$P$500,"Booked-Paid")</f>
         <v>3</v>
       </c>
-      <c r="F2" s="7" t="n">
+      <c r="F2" s="11" t="n">
         <f aca="false">SUMIFS('Referral Tracking'!$S$2:$S$500,'Referral Tracking'!$D$2:$D$500,A2)</f>
-        <v>4500</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2196,7 +2191,7 @@
         <f aca="false">COUNTIFS('Referral Tracking'!$D$2:$D$500,A3,'Referral Tracking'!$P$2:$P$500,"Booked-Paid")</f>
         <v>0</v>
       </c>
-      <c r="F3" s="7" t="n">
+      <c r="F3" s="11" t="n">
         <f aca="false">SUMIFS('Referral Tracking'!$S$2:$S$500,'Referral Tracking'!$D$2:$D$500,A3)</f>
         <v>0</v>
       </c>
@@ -2222,7 +2217,7 @@
         <f aca="false">COUNTIFS('Referral Tracking'!$D$2:$D$500,A4,'Referral Tracking'!$P$2:$P$500,"Booked-Paid")</f>
         <v>0</v>
       </c>
-      <c r="F4" s="7" t="n">
+      <c r="F4" s="11" t="n">
         <f aca="false">SUMIFS('Referral Tracking'!$S$2:$S$500,'Referral Tracking'!$D$2:$D$500,A4)</f>
         <v>0</v>
       </c>
@@ -2248,7 +2243,7 @@
         <f aca="false">COUNTIFS('Referral Tracking'!$D$2:$D$500,A5,'Referral Tracking'!$P$2:$P$500,"Booked-Paid")</f>
         <v>0</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="11" t="n">
         <f aca="false">SUMIFS('Referral Tracking'!$S$2:$S$500,'Referral Tracking'!$D$2:$D$500,A5)</f>
         <v>0</v>
       </c>
@@ -2274,7 +2269,7 @@
         <f aca="false">COUNTIFS('Referral Tracking'!$D$2:$D$500,A6,'Referral Tracking'!$P$2:$P$500,"Booked-Paid")</f>
         <v>0</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="11" t="n">
         <f aca="false">SUMIFS('Referral Tracking'!$S$2:$S$500,'Referral Tracking'!$D$2:$D$500,A6)</f>
         <v>0</v>
       </c>
@@ -2300,7 +2295,7 @@
         <f aca="false">COUNTIFS('Referral Tracking'!$D$2:$D$500,A7,'Referral Tracking'!$P$2:$P$500,"Booked-Paid")</f>
         <v>0</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="11" t="n">
         <f aca="false">SUMIFS('Referral Tracking'!$S$2:$S$500,'Referral Tracking'!$D$2:$D$500,A7)</f>
         <v>0</v>
       </c>
@@ -2326,7 +2321,7 @@
         <f aca="false">COUNTIFS('Referral Tracking'!$D$2:$D$500,A8,'Referral Tracking'!$P$2:$P$500,"Booked-Paid")</f>
         <v>0</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="11" t="n">
         <f aca="false">SUMIFS('Referral Tracking'!$S$2:$S$500,'Referral Tracking'!$D$2:$D$500,A8)</f>
         <v>0</v>
       </c>
@@ -2352,7 +2347,7 @@
         <f aca="false">COUNTIFS('Referral Tracking'!$D$2:$D$500,A9,'Referral Tracking'!$P$2:$P$500,"Booked-Paid")</f>
         <v>0</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="F9" s="11" t="n">
         <f aca="false">SUMIFS('Referral Tracking'!$S$2:$S$500,'Referral Tracking'!$D$2:$D$500,A9)</f>
         <v>0</v>
       </c>
@@ -2378,7 +2373,7 @@
         <f aca="false">COUNTIFS('Referral Tracking'!$D$2:$D$500,A10,'Referral Tracking'!$P$2:$P$500,"Booked-Paid")</f>
         <v>0</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="11" t="n">
         <f aca="false">SUMIFS('Referral Tracking'!$S$2:$S$500,'Referral Tracking'!$D$2:$D$500,A10)</f>
         <v>0</v>
       </c>
@@ -2404,20 +2399,20 @@
         <f aca="false">COUNTIFS('Referral Tracking'!$D$2:$D$500,A11,'Referral Tracking'!$P$2:$P$500,"Booked-Paid")</f>
         <v>0</v>
       </c>
-      <c r="F11" s="7" t="n">
+      <c r="F11" s="11" t="n">
         <f aca="false">SUMIFS('Referral Tracking'!$S$2:$S$500,'Referral Tracking'!$D$2:$D$500,A11)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2508,7 +2503,7 @@
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">SUMIF('Referral Tracking'!$T$2:$T$500,"Y",'Referral Tracking'!$S$2:$S$500)</f>
-        <v>4500</v>
+        <v>5900</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2519,7 +2514,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B11" s="15" t="n">
         <f aca="false">COUNTIF('Referral Tracking'!$C$2:$C$500,"Employee Pre-Submitted")</f>
@@ -2528,7 +2523,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B12" s="15" t="n">
         <f aca="false">COUNTIF('Referral Tracking'!$C$2:$C$500,"Client WhatsApp Form")</f>
@@ -2543,7 +2538,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B14" s="15" t="n">
         <f aca="false">COUNTIF('Referral Tracking'!$J$2:$J$500,"Sahel Reservation")</f>
@@ -2552,7 +2547,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B15" s="15" t="n">
         <f aca="false">COUNTIF('Referral Tracking'!$J$2:$J$500,"Furnishing Package")</f>

</xml_diff>